<commit_message>
Yayın: keşif özeti tenzilatlı fiyata çevrildi
Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HJPp6bx7wepUX5p8fxGcjg
</commit_message>
<xml_diff>
--- a/belgeler/15_KESIF_OZETLERI.xlsx
+++ b/belgeler/15_KESIF_OZETLERI.xlsx
@@ -1536,7 +1536,7 @@
         <v/>
       </c>
       <c r="I6" s="13" t="n">
-        <v>62.35</v>
+        <v>52.37</v>
       </c>
     </row>
     <row r="7" ht="22" customHeight="1">
@@ -1576,7 +1576,7 @@
         <v/>
       </c>
       <c r="I7" s="13" t="n">
-        <v>71.84999999999999</v>
+        <v>60.35</v>
       </c>
     </row>
     <row r="8" ht="33" customHeight="1">
@@ -1616,7 +1616,7 @@
         <v/>
       </c>
       <c r="I8" s="13" t="n">
-        <v>3274.35</v>
+        <v>2750.45</v>
       </c>
     </row>
     <row r="9" ht="33" customHeight="1">
@@ -1656,7 +1656,7 @@
         <v/>
       </c>
       <c r="I9" s="13" t="n">
-        <v>3524.35</v>
+        <v>2960.45</v>
       </c>
     </row>
     <row r="10" ht="14" customHeight="1">
@@ -1696,7 +1696,7 @@
         <v/>
       </c>
       <c r="I10" s="13" t="n">
-        <v>43987.5</v>
+        <v>36949.5</v>
       </c>
     </row>
     <row r="11" ht="22" customHeight="1">
@@ -1736,7 +1736,7 @@
         <v/>
       </c>
       <c r="I11" s="13" t="n">
-        <v>46482.43</v>
+        <v>39045.24</v>
       </c>
     </row>
     <row r="12" ht="22" customHeight="1">
@@ -1776,7 +1776,7 @@
         <v/>
       </c>
       <c r="I12" s="13" t="n">
-        <v>44681.18</v>
+        <v>37532.19</v>
       </c>
     </row>
     <row r="13" ht="22" customHeight="1">
@@ -1816,7 +1816,7 @@
         <v/>
       </c>
       <c r="I13" s="13" t="n">
-        <v>85943.50999999999</v>
+        <v>72192.55</v>
       </c>
     </row>
     <row r="14" ht="14" customHeight="1">
@@ -1856,7 +1856,7 @@
         <v/>
       </c>
       <c r="I14" s="13" t="n">
-        <v>1028.33</v>
+        <v>863.8</v>
       </c>
     </row>
     <row r="15" ht="22" customHeight="1">
@@ -1896,7 +1896,7 @@
         <v/>
       </c>
       <c r="I15" s="13" t="n">
-        <v>723.73</v>
+        <v>607.9299999999999</v>
       </c>
     </row>
     <row r="16" ht="22" customHeight="1">
@@ -1936,7 +1936,7 @@
         <v/>
       </c>
       <c r="I16" s="13" t="n">
-        <v>1106.28</v>
+        <v>929.28</v>
       </c>
     </row>
     <row r="17" ht="22" customHeight="1">
@@ -1976,7 +1976,7 @@
         <v/>
       </c>
       <c r="I17" s="13" t="n">
-        <v>2116.1</v>
+        <v>1777.52</v>
       </c>
     </row>
     <row r="18" ht="14" customHeight="1">
@@ -2016,7 +2016,7 @@
         <v/>
       </c>
       <c r="I18" s="13" t="n">
-        <v>443.51</v>
+        <v>372.55</v>
       </c>
     </row>
     <row r="19" ht="22" customHeight="1">
@@ -2056,7 +2056,7 @@
         <v/>
       </c>
       <c r="I19" s="13" t="n">
-        <v>454.16</v>
+        <v>381.49</v>
       </c>
     </row>
     <row r="20" ht="22" customHeight="1">
@@ -2096,7 +2096,7 @@
         <v/>
       </c>
       <c r="I20" s="13" t="n">
-        <v>296.13</v>
+        <v>248.75</v>
       </c>
     </row>
     <row r="21" ht="22" customHeight="1">
@@ -2136,7 +2136,7 @@
         <v/>
       </c>
       <c r="I21" s="13" t="n">
-        <v>386.03</v>
+        <v>324.27</v>
       </c>
     </row>
     <row r="22" ht="22" customHeight="1">
@@ -2176,7 +2176,7 @@
         <v/>
       </c>
       <c r="I22" s="13" t="n">
-        <v>218.54</v>
+        <v>183.57</v>
       </c>
     </row>
     <row r="23" ht="22" customHeight="1">
@@ -2216,7 +2216,7 @@
         <v/>
       </c>
       <c r="I23" s="13" t="n">
-        <v>175.8</v>
+        <v>147.67</v>
       </c>
     </row>
     <row r="24" ht="14" customHeight="1">
@@ -2256,7 +2256,7 @@
         <v/>
       </c>
       <c r="I24" s="13" t="n">
-        <v>4457.5</v>
+        <v>3744.3</v>
       </c>
     </row>
     <row r="25" ht="22" customHeight="1">
@@ -2296,7 +2296,7 @@
         <v/>
       </c>
       <c r="I25" s="13" t="n">
-        <v>49741.82</v>
+        <v>41783.13</v>
       </c>
     </row>
     <row r="26" ht="22" customHeight="1">
@@ -2336,7 +2336,7 @@
         <v/>
       </c>
       <c r="I26" s="13" t="n">
-        <v>12003.52</v>
+        <v>10082.96</v>
       </c>
     </row>
     <row r="27" ht="14" customHeight="1">
@@ -2376,7 +2376,7 @@
         <v/>
       </c>
       <c r="I27" s="13" t="n">
-        <v>13847.2</v>
+        <v>11631.65</v>
       </c>
     </row>
     <row r="28" ht="22" customHeight="1">
@@ -2416,7 +2416,7 @@
         <v/>
       </c>
       <c r="I28" s="13" t="n">
-        <v>5280.06</v>
+        <v>4435.25</v>
       </c>
     </row>
     <row r="29" ht="14" customHeight="1">
@@ -2456,7 +2456,7 @@
         <v/>
       </c>
       <c r="I29" s="13" t="n">
-        <v>7048.52</v>
+        <v>5920.76</v>
       </c>
     </row>
     <row r="30" ht="14" customHeight="1">
@@ -2496,7 +2496,7 @@
         <v/>
       </c>
       <c r="I30" s="13" t="n">
-        <v>1709.76</v>
+        <v>1436.2</v>
       </c>
     </row>
     <row r="31" ht="14" customHeight="1">
@@ -2536,7 +2536,7 @@
         <v/>
       </c>
       <c r="I31" s="13" t="n">
-        <v>53225.97</v>
+        <v>44709.81</v>
       </c>
     </row>
     <row r="32" ht="22" customHeight="1">
@@ -2576,7 +2576,7 @@
         <v/>
       </c>
       <c r="I32" s="13" t="n">
-        <v>2640.66</v>
+        <v>2218.15</v>
       </c>
     </row>
     <row r="33" ht="22" customHeight="1">
@@ -2616,7 +2616,7 @@
         <v/>
       </c>
       <c r="I33" s="13" t="n">
-        <v>223.96</v>
+        <v>188.13</v>
       </c>
     </row>
     <row r="34" ht="22" customHeight="1">
@@ -2656,7 +2656,7 @@
         <v/>
       </c>
       <c r="I34" s="13" t="n">
-        <v>84.91</v>
+        <v>71.31999999999999</v>
       </c>
     </row>
     <row r="35" ht="22" customHeight="1">
@@ -2696,7 +2696,7 @@
         <v/>
       </c>
       <c r="I35" s="13" t="n">
-        <v>290.5</v>
+        <v>244.02</v>
       </c>
     </row>
     <row r="36" ht="22" customHeight="1">
@@ -2736,7 +2736,7 @@
         <v/>
       </c>
       <c r="I36" s="13" t="n">
-        <v>395.44</v>
+        <v>332.17</v>
       </c>
     </row>
     <row r="37" ht="14" customHeight="1">
@@ -2776,7 +2776,7 @@
         <v/>
       </c>
       <c r="I37" s="13" t="n">
-        <v>28.05</v>
+        <v>23.56</v>
       </c>
     </row>
     <row r="38" ht="14" customHeight="1">
@@ -2816,7 +2816,7 @@
         <v/>
       </c>
       <c r="I38" s="13" t="n">
-        <v>39.41</v>
+        <v>33.1</v>
       </c>
     </row>
     <row r="39" ht="14" customHeight="1">
@@ -2856,7 +2856,7 @@
         <v/>
       </c>
       <c r="I39" s="13" t="n">
-        <v>88.59</v>
+        <v>74.42</v>
       </c>
     </row>
     <row r="40" ht="22" customHeight="1">
@@ -2896,7 +2896,7 @@
         <v/>
       </c>
       <c r="I40" s="13" t="n">
-        <v>1848.1</v>
+        <v>1552.4</v>
       </c>
     </row>
     <row r="41" ht="22" customHeight="1">
@@ -2936,7 +2936,7 @@
         <v/>
       </c>
       <c r="I41" s="13" t="n">
-        <v>2646.28</v>
+        <v>2222.88</v>
       </c>
     </row>
     <row r="42" ht="14" customHeight="1">
@@ -2976,7 +2976,7 @@
         <v/>
       </c>
       <c r="I42" s="13" t="n">
-        <v>9896.620000000001</v>
+        <v>8313.16</v>
       </c>
     </row>
     <row r="43" ht="22" customHeight="1">
@@ -3016,7 +3016,7 @@
         <v/>
       </c>
       <c r="I43" s="13" t="n">
-        <v>9265.620000000001</v>
+        <v>7783.12</v>
       </c>
     </row>
     <row r="44" ht="22" customHeight="1">
@@ -3056,7 +3056,7 @@
         <v/>
       </c>
       <c r="I44" s="13" t="n">
-        <v>576288.2</v>
+        <v>484082.09</v>
       </c>
     </row>
     <row r="45" ht="14" customHeight="1">
@@ -3096,7 +3096,7 @@
         <v/>
       </c>
       <c r="I45" s="13" t="n">
-        <v>99145.64999999999</v>
+        <v>83282.35000000001</v>
       </c>
     </row>
     <row r="46" ht="14" customHeight="1">
@@ -3136,7 +3136,7 @@
         <v/>
       </c>
       <c r="I46" s="13" t="n">
-        <v>20726.2</v>
+        <v>17410.01</v>
       </c>
     </row>
     <row r="47" ht="22" customHeight="1">
@@ -3176,7 +3176,7 @@
         <v/>
       </c>
       <c r="I47" s="13" t="n">
-        <v>572.8</v>
+        <v>481.15</v>
       </c>
     </row>
     <row r="48" ht="22" customHeight="1">
@@ -3216,7 +3216,7 @@
         <v/>
       </c>
       <c r="I48" s="13" t="n">
-        <v>185.85</v>
+        <v>156.11</v>
       </c>
     </row>
     <row r="49" ht="22" customHeight="1">
@@ -3256,7 +3256,7 @@
         <v/>
       </c>
       <c r="I49" s="13" t="n">
-        <v>393.69</v>
+        <v>330.7</v>
       </c>
     </row>
     <row r="50" ht="33" customHeight="1">
@@ -3296,7 +3296,7 @@
         <v/>
       </c>
       <c r="I50" s="13" t="n">
-        <v>1624.67</v>
+        <v>1364.72</v>
       </c>
     </row>
     <row r="51" ht="14" customHeight="1">
@@ -3336,7 +3336,7 @@
         <v/>
       </c>
       <c r="I51" s="13" t="n">
-        <v>1120.05</v>
+        <v>940.84</v>
       </c>
     </row>
     <row r="52" ht="14" customHeight="1">
@@ -3376,7 +3376,7 @@
         <v/>
       </c>
       <c r="I52" s="13" t="n">
-        <v>271.25</v>
+        <v>227.85</v>
       </c>
     </row>
     <row r="53" ht="33" customHeight="1">
@@ -3416,7 +3416,7 @@
         <v/>
       </c>
       <c r="I53" s="13" t="n">
-        <v>1035.88</v>
+        <v>870.14</v>
       </c>
     </row>
     <row r="54" ht="33" customHeight="1">
@@ -3456,7 +3456,7 @@
         <v/>
       </c>
       <c r="I54" s="13" t="n">
-        <v>3199.68</v>
+        <v>2687.73</v>
       </c>
     </row>
     <row r="55" ht="44" customHeight="1">
@@ -3496,7 +3496,7 @@
         <v/>
       </c>
       <c r="I55" s="13" t="n">
-        <v>835.1</v>
+        <v>701.48</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Yayın: keşif özetlerinden fiyat sütunu uyarısı kaldırıldı
Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HJPp6bx7wepUX5p8fxGcjg
</commit_message>
<xml_diff>
--- a/belgeler/15_KESIF_OZETLERI.xlsx
+++ b/belgeler/15_KESIF_OZETLERI.xlsx
@@ -827,13 +827,6 @@
         </is>
       </c>
     </row>
-    <row r="3">
-      <c r="A3" s="14" t="inlineStr">
-        <is>
-          <t>Bu keşif özeti yalnızca bu yapıya aittir. TKDK'ya sunulacak nüshada F ve G sütunları (birim fiyat ve tutar) gizlenmelidir; keşif özetinde fiyat sütunu bulunmaz.</t>
-        </is>
-      </c>
-    </row>
     <row r="5" ht="30" customHeight="1">
       <c r="A5" s="2" t="inlineStr">
         <is>
@@ -1380,12 +1373,11 @@
       </c>
     </row>
   </sheetData>
-  <mergeCells count="5">
+  <mergeCells count="4">
     <mergeCell ref="A13:A21"/>
+    <mergeCell ref="A11:A12"/>
+    <mergeCell ref="A2:G2"/>
     <mergeCell ref="A1:G1"/>
-    <mergeCell ref="A3:G3"/>
-    <mergeCell ref="A2:G2"/>
-    <mergeCell ref="A11:A12"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1422,7 +1414,7 @@
     <row r="2">
       <c r="A2" s="14" t="inlineStr">
         <is>
-          <t>Sarı hücreler değiştirilebilir. Fiyatlar keşif özetinin birimine göredir (dönüşümlü pozlarda ör. TL/kg, TL/m²) ve KDV hariçtir. Keşif özetinin TKDK'ya sunulan nüshasında fiyat sütunu bulunmaz; bu sekme kendi maliyet takibiniz içindir.</t>
+          <t>Sarı hücreler değiştirilebilir. Fiyatlar keşif özetinin birimine göredir (dönüşümlü pozlarda ör. TL/kg, TL/m²) ve KDV hariçtir.</t>
         </is>
       </c>
     </row>
@@ -3540,13 +3532,6 @@
         </is>
       </c>
     </row>
-    <row r="3">
-      <c r="A3" s="14" t="inlineStr">
-        <is>
-          <t>Bu keşif özeti yalnızca bu yapıya aittir. TKDK'ya sunulacak nüshada F ve G sütunları (birim fiyat ve tutar) gizlenmelidir; keşif özetinde fiyat sütunu bulunmaz.</t>
-        </is>
-      </c>
-    </row>
     <row r="5" ht="30" customHeight="1">
       <c r="A5" s="2" t="inlineStr">
         <is>
@@ -4788,12 +4773,11 @@
       </c>
     </row>
   </sheetData>
-  <mergeCells count="11">
+  <mergeCells count="10">
     <mergeCell ref="A1:G1"/>
     <mergeCell ref="A13:A14"/>
-    <mergeCell ref="A3:G3"/>
+    <mergeCell ref="A25:A26"/>
     <mergeCell ref="A10:A12"/>
-    <mergeCell ref="A25:A26"/>
     <mergeCell ref="A20:A22"/>
     <mergeCell ref="A15:A17"/>
     <mergeCell ref="A2:G2"/>
@@ -4837,13 +4821,6 @@
         </is>
       </c>
     </row>
-    <row r="3">
-      <c r="A3" s="14" t="inlineStr">
-        <is>
-          <t>Bu keşif özeti yalnızca bu yapıya aittir. TKDK'ya sunulacak nüshada F ve G sütunları (birim fiyat ve tutar) gizlenmelidir; keşif özetinde fiyat sütunu bulunmaz.</t>
-        </is>
-      </c>
-    </row>
     <row r="5" ht="30" customHeight="1">
       <c r="A5" s="2" t="inlineStr">
         <is>
@@ -6085,12 +6062,11 @@
       </c>
     </row>
   </sheetData>
-  <mergeCells count="11">
+  <mergeCells count="10">
     <mergeCell ref="A1:G1"/>
     <mergeCell ref="A13:A14"/>
-    <mergeCell ref="A3:G3"/>
+    <mergeCell ref="A25:A26"/>
     <mergeCell ref="A10:A12"/>
-    <mergeCell ref="A25:A26"/>
     <mergeCell ref="A20:A22"/>
     <mergeCell ref="A15:A17"/>
     <mergeCell ref="A2:G2"/>
@@ -6134,13 +6110,6 @@
         </is>
       </c>
     </row>
-    <row r="3">
-      <c r="A3" s="14" t="inlineStr">
-        <is>
-          <t>Bu keşif özeti yalnızca bu yapıya aittir. TKDK'ya sunulacak nüshada F ve G sütunları (birim fiyat ve tutar) gizlenmelidir; keşif özetinde fiyat sütunu bulunmaz.</t>
-        </is>
-      </c>
-    </row>
     <row r="5" ht="30" customHeight="1">
       <c r="A5" s="2" t="inlineStr">
         <is>
@@ -6389,9 +6358,8 @@
       </c>
     </row>
   </sheetData>
-  <mergeCells count="4">
+  <mergeCells count="3">
     <mergeCell ref="A10:A11"/>
-    <mergeCell ref="A3:G3"/>
     <mergeCell ref="A2:G2"/>
     <mergeCell ref="A1:G1"/>
   </mergeCells>
@@ -6431,13 +6399,6 @@
         </is>
       </c>
     </row>
-    <row r="3">
-      <c r="A3" s="14" t="inlineStr">
-        <is>
-          <t>Bu keşif özeti yalnızca bu yapıya aittir. TKDK'ya sunulacak nüshada F ve G sütunları (birim fiyat ve tutar) gizlenmelidir; keşif özetinde fiyat sütunu bulunmaz.</t>
-        </is>
-      </c>
-    </row>
     <row r="5" ht="30" customHeight="1">
       <c r="A5" s="2" t="inlineStr">
         <is>
@@ -6657,8 +6618,7 @@
       </c>
     </row>
   </sheetData>
-  <mergeCells count="3">
-    <mergeCell ref="A3:G3"/>
+  <mergeCells count="2">
     <mergeCell ref="A2:G2"/>
     <mergeCell ref="A1:G1"/>
   </mergeCells>
@@ -6698,13 +6658,6 @@
         </is>
       </c>
     </row>
-    <row r="3">
-      <c r="A3" s="14" t="inlineStr">
-        <is>
-          <t>Bu keşif özeti yalnızca bu yapıya aittir. TKDK'ya sunulacak nüshada F ve G sütunları (birim fiyat ve tutar) gizlenmelidir; keşif özetinde fiyat sütunu bulunmaz.</t>
-        </is>
-      </c>
-    </row>
     <row r="5" ht="30" customHeight="1">
       <c r="A5" s="2" t="inlineStr">
         <is>
@@ -6924,8 +6877,7 @@
       </c>
     </row>
   </sheetData>
-  <mergeCells count="3">
-    <mergeCell ref="A3:G3"/>
+  <mergeCells count="2">
     <mergeCell ref="A2:G2"/>
     <mergeCell ref="A1:G1"/>
   </mergeCells>
@@ -6965,13 +6917,6 @@
         </is>
       </c>
     </row>
-    <row r="3">
-      <c r="A3" s="14" t="inlineStr">
-        <is>
-          <t>Bu keşif özeti yalnızca bu yapıya aittir. TKDK'ya sunulacak nüshada F ve G sütunları (birim fiyat ve tutar) gizlenmelidir; keşif özetinde fiyat sütunu bulunmaz.</t>
-        </is>
-      </c>
-    </row>
     <row r="5" ht="30" customHeight="1">
       <c r="A5" s="2" t="inlineStr">
         <is>
@@ -7191,8 +7136,7 @@
       </c>
     </row>
   </sheetData>
-  <mergeCells count="3">
-    <mergeCell ref="A3:G3"/>
+  <mergeCells count="2">
     <mergeCell ref="A2:G2"/>
     <mergeCell ref="A1:G1"/>
   </mergeCells>
@@ -7232,13 +7176,6 @@
         </is>
       </c>
     </row>
-    <row r="3">
-      <c r="A3" s="14" t="inlineStr">
-        <is>
-          <t>Bu keşif özeti yalnızca bu yapıya aittir. TKDK'ya sunulacak nüshada F ve G sütunları (birim fiyat ve tutar) gizlenmelidir; keşif özetinde fiyat sütunu bulunmaz.</t>
-        </is>
-      </c>
-    </row>
     <row r="5" ht="30" customHeight="1">
       <c r="A5" s="2" t="inlineStr">
         <is>
@@ -7458,8 +7395,7 @@
       </c>
     </row>
   </sheetData>
-  <mergeCells count="3">
-    <mergeCell ref="A3:G3"/>
+  <mergeCells count="2">
     <mergeCell ref="A2:G2"/>
     <mergeCell ref="A1:G1"/>
   </mergeCells>

</xml_diff>